<commit_message>
Waiting for Asset workflow changes
</commit_message>
<xml_diff>
--- a/src/test/resources/data/stibo.xlsx
+++ b/src/test/resources/data/stibo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\AK1PEPF00000206\EXCELCNV\399f3ce1-9b24-468f-9bff-ded1a8751bdd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95AD653F-6755-42CE-A2DD-C6A15A9D88E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{885053A4-5FDB-441D-A1FD-41B698C1438C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" firstSheet="1" activeTab="1" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" firstSheet="1" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
   </bookViews>
   <sheets>
     <sheet name="consignment" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="147">
   <si>
     <t>ID</t>
   </si>
@@ -243,10 +243,10 @@
     <t>Singles per Outer TC</t>
   </si>
   <si>
-    <t>PRD0117-A</t>
-  </si>
-  <si>
-    <t>PRD0117</t>
+    <t>PRD0123-A</t>
+  </si>
+  <si>
+    <t>PRD0123</t>
   </si>
   <si>
     <t>100% FAKE</t>
@@ -330,6 +330,9 @@
     <t>Knee length</t>
   </si>
   <si>
+    <t>5056875531106</t>
+  </si>
+  <si>
     <t>WHITE</t>
   </si>
   <si>
@@ -348,7 +351,7 @@
     <t>pic.png</t>
   </si>
   <si>
-    <t>Consignment_Supplier_PRD0117</t>
+    <t>Consignment_Supplier_PRD0123</t>
   </si>
   <si>
     <t>SSALT CLOTHING / JOGGERS (INT.L6-G8-T8310F)</t>
@@ -387,37 +390,52 @@
     <t>MSS101 (590x380x380)</t>
   </si>
   <si>
-    <t>PRD0117-B</t>
+    <t>PRD0123-B</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>PRD0118-A</t>
-  </si>
-  <si>
-    <t>PRD0118</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0118</t>
-  </si>
-  <si>
-    <t>PRD0118-B</t>
+    <t>5056875531137</t>
+  </si>
+  <si>
+    <t>PRD0124-A</t>
+  </si>
+  <si>
+    <t>PRD0124</t>
+  </si>
+  <si>
+    <t>5056831829018</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0124</t>
+  </si>
+  <si>
+    <t>PRD0124-B</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>PRD0119-A</t>
-  </si>
-  <si>
-    <t>PRD0119</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0119</t>
-  </si>
-  <si>
-    <t>PRD0119-B</t>
+    <t>5056875531113</t>
+  </si>
+  <si>
+    <t>PRD0125-A</t>
+  </si>
+  <si>
+    <t>PRD0125</t>
+  </si>
+  <si>
+    <t>5056831829056</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0125</t>
+  </si>
+  <si>
+    <t>PRD0125-B</t>
+  </si>
+  <si>
+    <t>5056875531168</t>
   </si>
   <si>
     <t>Catagory</t>
@@ -591,7 +609,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1413,56 +1431,56 @@
       <c r="AH2" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI2" s="10">
-        <v>5056875531083</v>
+      <c r="AI2" s="10" t="s">
+        <v>97</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL2" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN2" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP2" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ2" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR2" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AS2" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT2" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU2" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV2" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW2" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX2" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY2" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ2" s="1">
         <v>25</v>
@@ -1471,22 +1489,22 @@
         <v>20</v>
       </c>
       <c r="BB2" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC2" s="1" t="s">
         <v>69</v>
       </c>
       <c r="BD2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE2" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH2" s="1" t="s">
         <v>82</v>
@@ -1504,10 +1522,10 @@
         <v>100</v>
       </c>
       <c r="BM2" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN2" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO2" s="1">
         <v>100</v>
@@ -1525,7 +1543,7 @@
         <v>100</v>
       </c>
       <c r="BT2" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU2" s="1">
         <v>100</v>
@@ -1533,7 +1551,7 @@
     </row>
     <row r="3" spans="1:73">
       <c r="A3" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>69</v>
@@ -1605,7 +1623,7 @@
         <v>87</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>89</v>
@@ -1634,56 +1652,56 @@
       <c r="AH3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI3" s="10">
-        <v>5056831829032</v>
+      <c r="AI3" s="10" t="s">
+        <v>119</v>
       </c>
       <c r="AJ3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL3" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL3" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM3" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ3" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR3" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AS3" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT3" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU3" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV3" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW3" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX3" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY3" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ3" s="1">
         <v>25</v>
@@ -1692,22 +1710,22 @@
         <v>20</v>
       </c>
       <c r="BB3" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC3" s="1" t="s">
         <v>69</v>
       </c>
       <c r="BD3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE3" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG3" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH3" s="1" t="s">
         <v>82</v>
@@ -1725,10 +1743,10 @@
         <v>100</v>
       </c>
       <c r="BM3" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN3" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO3" s="1">
         <v>100</v>
@@ -1746,7 +1764,7 @@
         <v>100</v>
       </c>
       <c r="BT3" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU3" s="1">
         <v>100</v>
@@ -1754,13 +1772,13 @@
     </row>
     <row r="4" spans="1:73">
       <c r="A4" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>70</v>
@@ -1855,56 +1873,56 @@
       <c r="AH4" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI4" s="10">
-        <v>5056831828998</v>
+      <c r="AI4" s="10" t="s">
+        <v>122</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL4" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL4" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM4" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ4" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR4" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="AS4" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT4" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU4" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW4" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX4" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY4" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ4" s="1">
         <v>25</v>
@@ -1913,22 +1931,22 @@
         <v>20</v>
       </c>
       <c r="BB4" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC4" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="BD4" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE4" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF4" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG4" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH4" s="1" t="s">
         <v>82</v>
@@ -1946,10 +1964,10 @@
         <v>100</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO4" s="1">
         <v>100</v>
@@ -1967,7 +1985,7 @@
         <v>100</v>
       </c>
       <c r="BT4" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU4" s="1">
         <v>100</v>
@@ -1975,13 +1993,13 @@
     </row>
     <row r="5" spans="1:73">
       <c r="A5" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>70</v>
@@ -2047,7 +2065,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>89</v>
@@ -2076,56 +2094,56 @@
       <c r="AH5" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI5" s="10">
-        <v>5056875531120</v>
+      <c r="AI5" s="10" t="s">
+        <v>126</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL5" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM5" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ5" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR5" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="AS5" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT5" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU5" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV5" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW5" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX5" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY5" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ5" s="1">
         <v>25</v>
@@ -2134,22 +2152,22 @@
         <v>20</v>
       </c>
       <c r="BB5" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC5" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="BD5" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE5" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF5" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG5" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH5" s="1" t="s">
         <v>82</v>
@@ -2167,10 +2185,10 @@
         <v>100</v>
       </c>
       <c r="BM5" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN5" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO5" s="1">
         <v>100</v>
@@ -2188,7 +2206,7 @@
         <v>100</v>
       </c>
       <c r="BT5" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU5" s="1">
         <v>100</v>
@@ -2196,13 +2214,13 @@
     </row>
     <row r="6" spans="1:73">
       <c r="A6" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>70</v>
@@ -2297,56 +2315,56 @@
       <c r="AH6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI6" s="10">
-        <v>5056831828974</v>
+      <c r="AI6" s="10" t="s">
+        <v>129</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK6" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL6" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM6" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ6" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR6" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="AS6" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT6" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU6" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV6" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW6" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX6" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY6" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ6" s="1">
         <v>25</v>
@@ -2355,22 +2373,22 @@
         <v>20</v>
       </c>
       <c r="BB6" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC6" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="BD6" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE6" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF6" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG6" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH6" s="1" t="s">
         <v>82</v>
@@ -2388,10 +2406,10 @@
         <v>100</v>
       </c>
       <c r="BM6" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN6" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO6" s="1">
         <v>100</v>
@@ -2409,7 +2427,7 @@
         <v>100</v>
       </c>
       <c r="BT6" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU6" s="1">
         <v>100</v>
@@ -2417,13 +2435,13 @@
     </row>
     <row r="7" spans="1:73">
       <c r="A7" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>70</v>
@@ -2489,7 +2507,7 @@
         <v>87</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>89</v>
@@ -2518,56 +2536,56 @@
       <c r="AH7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI7" s="10">
-        <v>5056875531090</v>
+      <c r="AI7" s="10" t="s">
+        <v>132</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AK7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL7" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AL7" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="AM7" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AQ7" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AR7" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="AS7" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT7" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU7" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV7" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AW7" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AX7" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AY7" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AZ7" s="1">
         <v>25</v>
@@ -2576,22 +2594,22 @@
         <v>20</v>
       </c>
       <c r="BB7" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BC7" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="BD7" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BE7" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BF7" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BG7" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BH7" s="1" t="s">
         <v>82</v>
@@ -2609,10 +2627,10 @@
         <v>100</v>
       </c>
       <c r="BM7" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BN7" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BO7" s="1">
         <v>100</v>
@@ -2630,7 +2648,7 @@
         <v>100</v>
       </c>
       <c r="BT7" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BU7" s="1">
         <v>100</v>
@@ -2842,7 +2860,7 @@
         <v>39</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>42</v>
@@ -2922,13 +2940,13 @@
     </row>
     <row r="2" spans="1:67">
       <c r="A2" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>70</v>
@@ -2937,7 +2955,7 @@
         <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>72</v>
@@ -2949,7 +2967,7 @@
         <v>74</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>76</v>
@@ -2964,10 +2982,10 @@
         <v>79</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>80</v>
@@ -2994,7 +3012,7 @@
         <v>87</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>89</v>
@@ -3027,55 +3045,55 @@
         <v>5063159279999</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="AO2" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AP2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AQ2" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="AR2" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="AS2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AT2" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AU2" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AV2" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AW2" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="AX2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AY2" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AZ2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BA2" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="BB2" s="1" t="s">
         <v>82</v>
@@ -3093,10 +3111,10 @@
         <v>100</v>
       </c>
       <c r="BG2" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BH2" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BI2" s="1">
         <v>100</v>
@@ -3114,7 +3132,7 @@
         <v>100</v>
       </c>
       <c r="BN2" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BO2" s="1">
         <v>100</v>
@@ -3122,13 +3140,13 @@
     </row>
     <row r="3" spans="1:67">
       <c r="A3" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>70</v>
@@ -3137,7 +3155,7 @@
         <v>71</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>72</v>
@@ -3149,7 +3167,7 @@
         <v>74</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>76</v>
@@ -3164,10 +3182,10 @@
         <v>79</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>80</v>
@@ -3194,7 +3212,7 @@
         <v>87</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>89</v>
@@ -3227,37 +3245,37 @@
         <v>5063160372115</v>
       </c>
       <c r="AK3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AL3" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AM3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AN3" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="AO3" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AQ3" s="1" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="AX3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AY3" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AZ3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="BA3" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="BB3" s="1" t="s">
         <v>82</v>
@@ -3275,10 +3293,10 @@
         <v>101</v>
       </c>
       <c r="BG3" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BH3" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BI3" s="1">
         <v>101</v>
@@ -3296,7 +3314,7 @@
         <v>101</v>
       </c>
       <c r="BN3" s="1" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="BO3" s="1">
         <v>101</v>

</xml_diff>

<commit_message>
E2E Success - Waiting for Asset workflow
</commit_message>
<xml_diff>
--- a/src/test/resources/data/stibo.xlsx
+++ b/src/test/resources/data/stibo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\AK1PEPF00000206\EXCELCNV\399f3ce1-9b24-468f-9bff-ded1a8751bdd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1ECA754-33D5-41D8-9683-5BAB5DD28500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{276B2283-C209-4D6B-926F-724CE8770B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
   </bookViews>
@@ -243,10 +243,10 @@
     <t>Singles per Outer TC</t>
   </si>
   <si>
-    <t>PRD0126-A</t>
-  </si>
-  <si>
-    <t>PRD0126</t>
+    <t>PRD0129-A</t>
+  </si>
+  <si>
+    <t>PRD0129</t>
   </si>
   <si>
     <t>100% FAKE</t>
@@ -330,7 +330,7 @@
     <t>Knee length</t>
   </si>
   <si>
-    <t>5056831828981</t>
+    <t>5056831830144</t>
   </si>
   <si>
     <t>WHITE</t>
@@ -351,7 +351,7 @@
     <t>pic.png</t>
   </si>
   <si>
-    <t>Consignment_Supplier_PRD0126</t>
+    <t>Consignment_Supplier_PRD0129</t>
   </si>
   <si>
     <t>SSALT CLOTHING / JOGGERS (INT.L6-G8-T8310F)</t>
@@ -390,52 +390,52 @@
     <t>MSS101 (590x380x380)</t>
   </si>
   <si>
-    <t>PRD0126-B</t>
+    <t>PRD0129-B</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>5056875531151</t>
-  </si>
-  <si>
-    <t>PRD0127-A</t>
-  </si>
-  <si>
-    <t>PRD0127</t>
-  </si>
-  <si>
-    <t>5056875531182</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0127</t>
-  </si>
-  <si>
-    <t>PRD0127-B</t>
+    <t>5056831829667</t>
+  </si>
+  <si>
+    <t>PRD0130-A</t>
+  </si>
+  <si>
+    <t>PRD0130</t>
+  </si>
+  <si>
+    <t>5056831830113</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0130</t>
+  </si>
+  <si>
+    <t>PRD0130-B</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>5056831829001</t>
-  </si>
-  <si>
-    <t>PRD0128-A</t>
-  </si>
-  <si>
-    <t>PRD0128</t>
-  </si>
-  <si>
-    <t>5056875531069</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0128</t>
-  </si>
-  <si>
-    <t>PRD0128-B</t>
-  </si>
-  <si>
-    <t>5056875531199</t>
+    <t>5056831829124</t>
+  </si>
+  <si>
+    <t>PRD0131-A</t>
+  </si>
+  <si>
+    <t>PRD0131</t>
+  </si>
+  <si>
+    <t>5056831829155</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0131</t>
+  </si>
+  <si>
+    <t>PRD0131-B</t>
+  </si>
+  <si>
+    <t>5056831829629</t>
   </si>
   <si>
     <t>Catagory</t>

</xml_diff>

<commit_message>
Waiting for Asset changes in test data
</commit_message>
<xml_diff>
--- a/src/test/resources/data/stibo.xlsx
+++ b/src/test/resources/data/stibo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\AK1PEPF00000206\EXCELCNV\399f3ce1-9b24-468f-9bff-ded1a8751bdd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{276B2283-C209-4D6B-926F-724CE8770B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FF5416B-E6AF-4CDB-AA69-064A7AEB9A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="148">
   <si>
     <t>ID</t>
   </si>
@@ -243,10 +243,10 @@
     <t>Singles per Outer TC</t>
   </si>
   <si>
-    <t>PRD0129-A</t>
-  </si>
-  <si>
-    <t>PRD0129</t>
+    <t>PRD0138-A</t>
+  </si>
+  <si>
+    <t>PRD0138</t>
   </si>
   <si>
     <t>100% FAKE</t>
@@ -330,7 +330,7 @@
     <t>Knee length</t>
   </si>
   <si>
-    <t>5056831830144</t>
+    <t>5056831829117</t>
   </si>
   <si>
     <t>WHITE</t>
@@ -351,7 +351,7 @@
     <t>pic.png</t>
   </si>
   <si>
-    <t>Consignment_Supplier_PRD0129</t>
+    <t>Consignment_Supplier_PRD0138</t>
   </si>
   <si>
     <t>SSALT CLOTHING / JOGGERS (INT.L6-G8-T8310F)</t>
@@ -390,52 +390,55 @@
     <t>MSS101 (590x380x380)</t>
   </si>
   <si>
-    <t>PRD0129-B</t>
+    <t>PRD0138-B</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>5056831829667</t>
-  </si>
-  <si>
-    <t>PRD0130-A</t>
-  </si>
-  <si>
-    <t>PRD0130</t>
-  </si>
-  <si>
-    <t>5056831830113</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0130</t>
-  </si>
-  <si>
-    <t>PRD0130-B</t>
+    <t>5056831829674</t>
+  </si>
+  <si>
+    <t>PRD0139-A</t>
+  </si>
+  <si>
+    <t>PRD0139</t>
+  </si>
+  <si>
+    <t>5056831829148</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0139</t>
+  </si>
+  <si>
+    <t>PRD0139-B</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>5056831829124</t>
-  </si>
-  <si>
-    <t>PRD0131-A</t>
-  </si>
-  <si>
-    <t>PRD0131</t>
-  </si>
-  <si>
-    <t>5056831829155</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0131</t>
-  </si>
-  <si>
-    <t>PRD0131-B</t>
-  </si>
-  <si>
-    <t>5056831829629</t>
+    <t>5056831830106</t>
+  </si>
+  <si>
+    <t>PRD0140-A</t>
+  </si>
+  <si>
+    <t>PRD0140</t>
+  </si>
+  <si>
+    <t>5056831829650</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0140</t>
+  </si>
+  <si>
+    <t>PRD0140-B</t>
+  </si>
+  <si>
+    <t>5056831829087</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
   <si>
     <t>Catagory</t>
@@ -1012,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF65416-6E79-4376-BC7D-B07D4E2F8EDC}">
-  <dimension ref="A1:BU7"/>
+  <dimension ref="A1:BU9"/>
   <sheetFormatPr defaultColWidth="7.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -2654,6 +2657,11 @@
         <v>100</v>
       </c>
     </row>
+    <row r="9" spans="1:73">
+      <c r="AR9" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555551" footer="0.51180555555555551"/>
@@ -2860,7 +2868,7 @@
         <v>39</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>42</v>
@@ -2940,13 +2948,13 @@
     </row>
     <row r="2" spans="1:67">
       <c r="A2" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>70</v>
@@ -2955,7 +2963,7 @@
         <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>72</v>
@@ -2967,7 +2975,7 @@
         <v>74</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>76</v>
@@ -2982,10 +2990,10 @@
         <v>79</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>80</v>
@@ -3012,7 +3020,7 @@
         <v>87</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>89</v>
@@ -3054,7 +3062,7 @@
         <v>98</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AO2" s="1" t="s">
         <v>82</v>
@@ -3063,10 +3071,10 @@
         <v>101</v>
       </c>
       <c r="AQ2" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AR2" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="AS2" t="s">
         <v>105</v>
@@ -3081,7 +3089,7 @@
         <v>112</v>
       </c>
       <c r="AW2" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AX2" s="1" t="s">
         <v>98</v>
@@ -3093,7 +3101,7 @@
         <v>98</v>
       </c>
       <c r="BA2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="BB2" s="1" t="s">
         <v>82</v>
@@ -3140,13 +3148,13 @@
     </row>
     <row r="3" spans="1:67">
       <c r="A3" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>70</v>
@@ -3155,7 +3163,7 @@
         <v>71</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>72</v>
@@ -3167,7 +3175,7 @@
         <v>74</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>76</v>
@@ -3182,10 +3190,10 @@
         <v>79</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>80</v>
@@ -3254,7 +3262,7 @@
         <v>98</v>
       </c>
       <c r="AN3" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AO3" s="1" t="s">
         <v>82</v>
@@ -3263,7 +3271,7 @@
         <v>101</v>
       </c>
       <c r="AQ3" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AX3" s="1" t="s">
         <v>98</v>
@@ -3275,7 +3283,7 @@
         <v>98</v>
       </c>
       <c r="BA3" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="BB3" s="1" t="s">
         <v>82</v>
@@ -3314,7 +3322,7 @@
         <v>101</v>
       </c>
       <c r="BN3" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="BO3" s="1">
         <v>101</v>

</xml_diff>

<commit_message>
test commit from MDS
</commit_message>
<xml_diff>
--- a/src/test/resources/data/stibo.xlsx
+++ b/src/test/resources/data/stibo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\AK1PEPF00000206\EXCELCNV\399f3ce1-9b24-468f-9bff-ded1a8751bdd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FF5416B-E6AF-4CDB-AA69-064A7AEB9A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95AD653F-6755-42CE-A2DD-C6A15A9D88E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="658" firstSheet="1" activeTab="1" xr2:uid="{B5FD9A40-D110-4867-9C3F-9BA3AB9A9875}"/>
   </bookViews>
   <sheets>
     <sheet name="consignment" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="141">
   <si>
     <t>ID</t>
   </si>
@@ -243,10 +243,10 @@
     <t>Singles per Outer TC</t>
   </si>
   <si>
-    <t>PRD0138-A</t>
-  </si>
-  <si>
-    <t>PRD0138</t>
+    <t>PRD0117-A</t>
+  </si>
+  <si>
+    <t>PRD0117</t>
   </si>
   <si>
     <t>100% FAKE</t>
@@ -330,9 +330,6 @@
     <t>Knee length</t>
   </si>
   <si>
-    <t>5056831829117</t>
-  </si>
-  <si>
     <t>WHITE</t>
   </si>
   <si>
@@ -351,7 +348,7 @@
     <t>pic.png</t>
   </si>
   <si>
-    <t>Consignment_Supplier_PRD0138</t>
+    <t>Consignment_Supplier_PRD0117</t>
   </si>
   <si>
     <t>SSALT CLOTHING / JOGGERS (INT.L6-G8-T8310F)</t>
@@ -390,55 +387,37 @@
     <t>MSS101 (590x380x380)</t>
   </si>
   <si>
-    <t>PRD0138-B</t>
+    <t>PRD0117-B</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>5056831829674</t>
-  </si>
-  <si>
-    <t>PRD0139-A</t>
-  </si>
-  <si>
-    <t>PRD0139</t>
-  </si>
-  <si>
-    <t>5056831829148</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0139</t>
-  </si>
-  <si>
-    <t>PRD0139-B</t>
+    <t>PRD0118-A</t>
+  </si>
+  <si>
+    <t>PRD0118</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0118</t>
+  </si>
+  <si>
+    <t>PRD0118-B</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>5056831830106</t>
-  </si>
-  <si>
-    <t>PRD0140-A</t>
-  </si>
-  <si>
-    <t>PRD0140</t>
-  </si>
-  <si>
-    <t>5056831829650</t>
-  </si>
-  <si>
-    <t>Consignment_Supplier_PRD0140</t>
-  </si>
-  <si>
-    <t>PRD0140-B</t>
-  </si>
-  <si>
-    <t>5056831829087</t>
-  </si>
-  <si>
-    <t>`</t>
+    <t>PRD0119-A</t>
+  </si>
+  <si>
+    <t>PRD0119</t>
+  </si>
+  <si>
+    <t>Consignment_Supplier_PRD0119</t>
+  </si>
+  <si>
+    <t>PRD0119-B</t>
   </si>
   <si>
     <t>Catagory</t>
@@ -612,7 +591,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1015,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF65416-6E79-4376-BC7D-B07D4E2F8EDC}">
-  <dimension ref="A1:BU9"/>
+  <dimension ref="A1:BU7"/>
   <sheetFormatPr defaultColWidth="7.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1434,56 +1413,56 @@
       <c r="AH2" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI2" s="10" t="s">
+      <c r="AI2" s="10">
+        <v>5056875531083</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AJ2" s="1" t="s">
+      <c r="AK2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK2" s="1" t="s">
+      <c r="AL2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM2" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL2" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM2" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN2" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP2" s="1" t="s">
+      <c r="AQ2" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ2" s="1" t="s">
+      <c r="AR2" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AS2" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="AS2" s="1" t="s">
+      <c r="AT2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT2" s="1" t="s">
+      <c r="AU2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU2" s="1" t="s">
+      <c r="AV2" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV2" s="1" t="s">
+      <c r="AW2" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW2" s="1" t="s">
+      <c r="AX2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX2" s="1" t="s">
+      <c r="AY2" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY2" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ2" s="1">
         <v>25</v>
@@ -1492,22 +1471,22 @@
         <v>20</v>
       </c>
       <c r="BB2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="BC2" s="1" t="s">
         <v>69</v>
       </c>
       <c r="BD2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BE2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="BF2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG2" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH2" s="1" t="s">
         <v>82</v>
@@ -1525,28 +1504,28 @@
         <v>100</v>
       </c>
       <c r="BM2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN2" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN2" s="1" t="s">
+      <c r="BO2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT2" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BO2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT2" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BU2" s="1">
         <v>100</v>
@@ -1554,7 +1533,7 @@
     </row>
     <row r="3" spans="1:73">
       <c r="A3" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>69</v>
@@ -1626,7 +1605,7 @@
         <v>87</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>89</v>
@@ -1655,56 +1634,56 @@
       <c r="AH3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI3" s="10" t="s">
-        <v>119</v>
+      <c r="AI3" s="10">
+        <v>5056831829032</v>
       </c>
       <c r="AJ3" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AK3" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK3" s="1" t="s">
+      <c r="AL3" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM3" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM3" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO3" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP3" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP3" s="1" t="s">
+      <c r="AQ3" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ3" s="1" t="s">
+      <c r="AR3" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AR3" s="1" t="s">
+      <c r="AS3" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="AS3" s="1" t="s">
+      <c r="AT3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT3" s="1" t="s">
+      <c r="AU3" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU3" s="1" t="s">
+      <c r="AV3" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV3" s="1" t="s">
+      <c r="AW3" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW3" s="1" t="s">
+      <c r="AX3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX3" s="1" t="s">
+      <c r="AY3" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY3" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ3" s="1">
         <v>25</v>
@@ -1713,22 +1692,22 @@
         <v>20</v>
       </c>
       <c r="BB3" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="BC3" s="1" t="s">
         <v>69</v>
       </c>
       <c r="BD3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BE3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="BF3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG3" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH3" s="1" t="s">
         <v>82</v>
@@ -1746,28 +1725,28 @@
         <v>100</v>
       </c>
       <c r="BM3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN3" s="1" t="s">
+      <c r="BO3" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP3" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ3" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR3" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS3" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT3" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BO3" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP3" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ3" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR3" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS3" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT3" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BU3" s="1">
         <v>100</v>
@@ -1775,13 +1754,13 @@
     </row>
     <row r="4" spans="1:73">
       <c r="A4" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>70</v>
@@ -1876,56 +1855,56 @@
       <c r="AH4" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI4" s="10" t="s">
-        <v>122</v>
+      <c r="AI4" s="10">
+        <v>5056831828998</v>
       </c>
       <c r="AJ4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AK4" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK4" s="1" t="s">
+      <c r="AL4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM4" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL4" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM4" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP4" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP4" s="1" t="s">
+      <c r="AQ4" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ4" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="AR4" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="AS4" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AT4" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT4" s="1" t="s">
+      <c r="AU4" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AV4" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AW4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW4" s="1" t="s">
+      <c r="AX4" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX4" s="1" t="s">
+      <c r="AY4" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY4" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ4" s="1">
         <v>25</v>
@@ -1934,22 +1913,22 @@
         <v>20</v>
       </c>
       <c r="BB4" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BC4" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="BD4" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="BE4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BC4" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="BD4" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BE4" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="BF4" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG4" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH4" s="1" t="s">
         <v>82</v>
@@ -1967,28 +1946,28 @@
         <v>100</v>
       </c>
       <c r="BM4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BO4" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP4" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ4" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR4" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS4" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT4" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BO4" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP4" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ4" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR4" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS4" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT4" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BU4" s="1">
         <v>100</v>
@@ -1996,13 +1975,13 @@
     </row>
     <row r="5" spans="1:73">
       <c r="A5" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>70</v>
@@ -2068,7 +2047,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>89</v>
@@ -2097,56 +2076,56 @@
       <c r="AH5" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI5" s="10" t="s">
-        <v>126</v>
+      <c r="AI5" s="10">
+        <v>5056875531120</v>
       </c>
       <c r="AJ5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AK5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK5" s="1" t="s">
+      <c r="AL5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM5" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM5" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO5" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP5" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP5" s="1" t="s">
+      <c r="AQ5" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ5" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="AR5" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="AS5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AT5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT5" s="1" t="s">
+      <c r="AU5" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU5" s="1" t="s">
+      <c r="AV5" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV5" s="1" t="s">
+      <c r="AW5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW5" s="1" t="s">
+      <c r="AX5" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX5" s="1" t="s">
+      <c r="AY5" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY5" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ5" s="1">
         <v>25</v>
@@ -2155,22 +2134,22 @@
         <v>20</v>
       </c>
       <c r="BB5" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BC5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="BD5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="BE5" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BC5" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="BD5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BE5" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="BF5" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG5" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH5" s="1" t="s">
         <v>82</v>
@@ -2188,28 +2167,28 @@
         <v>100</v>
       </c>
       <c r="BM5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN5" s="1" t="s">
+      <c r="BO5" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP5" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ5" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR5" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS5" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT5" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BO5" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP5" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ5" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR5" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS5" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT5" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BU5" s="1">
         <v>100</v>
@@ -2217,13 +2196,13 @@
     </row>
     <row r="6" spans="1:73">
       <c r="A6" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>70</v>
@@ -2318,56 +2297,56 @@
       <c r="AH6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI6" s="10" t="s">
-        <v>129</v>
+      <c r="AI6" s="10">
+        <v>5056831828974</v>
       </c>
       <c r="AJ6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AK6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK6" s="1" t="s">
+      <c r="AL6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM6" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL6" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM6" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO6" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP6" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP6" s="1" t="s">
+      <c r="AQ6" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ6" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="AR6" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="AS6" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AT6" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT6" s="1" t="s">
+      <c r="AU6" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU6" s="1" t="s">
+      <c r="AV6" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV6" s="1" t="s">
+      <c r="AW6" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW6" s="1" t="s">
+      <c r="AX6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX6" s="1" t="s">
+      <c r="AY6" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY6" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ6" s="1">
         <v>25</v>
@@ -2376,22 +2355,22 @@
         <v>20</v>
       </c>
       <c r="BB6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BC6" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="BD6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="BE6" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BC6" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="BD6" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BE6" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="BF6" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG6" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH6" s="1" t="s">
         <v>82</v>
@@ -2409,28 +2388,28 @@
         <v>100</v>
       </c>
       <c r="BM6" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN6" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN6" s="1" t="s">
+      <c r="BO6" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP6" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ6" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR6" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS6" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT6" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BO6" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP6" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ6" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR6" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS6" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT6" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BU6" s="1">
         <v>100</v>
@@ -2438,13 +2417,13 @@
     </row>
     <row r="7" spans="1:73">
       <c r="A7" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>70</v>
@@ -2510,7 +2489,7 @@
         <v>87</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>89</v>
@@ -2539,56 +2518,56 @@
       <c r="AH7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AI7" s="10" t="s">
-        <v>132</v>
+      <c r="AI7" s="10">
+        <v>5056875531090</v>
       </c>
       <c r="AJ7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AK7" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AK7" s="1" t="s">
+      <c r="AL7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM7" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="AL7" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AM7" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AO7" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP7" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AP7" s="1" t="s">
+      <c r="AQ7" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AQ7" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="AR7" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="AS7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AT7" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT7" s="1" t="s">
+      <c r="AU7" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU7" s="1" t="s">
+      <c r="AV7" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AV7" s="1" t="s">
+      <c r="AW7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AW7" s="1" t="s">
+      <c r="AX7" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AX7" s="1" t="s">
+      <c r="AY7" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="AY7" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="AZ7" s="1">
         <v>25</v>
@@ -2597,22 +2576,22 @@
         <v>20</v>
       </c>
       <c r="BB7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BC7" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="BD7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="BE7" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="BC7" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="BD7" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BE7" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="BF7" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BG7" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="BH7" s="1" t="s">
         <v>82</v>
@@ -2630,36 +2609,31 @@
         <v>100</v>
       </c>
       <c r="BM7" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BN7" s="1" t="s">
+      <c r="BO7" s="1">
+        <v>100</v>
+      </c>
+      <c r="BP7" s="1">
+        <v>100</v>
+      </c>
+      <c r="BQ7" s="1">
+        <v>100</v>
+      </c>
+      <c r="BR7" s="1">
+        <v>100</v>
+      </c>
+      <c r="BS7" s="1">
+        <v>100</v>
+      </c>
+      <c r="BT7" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="BO7" s="1">
-        <v>100</v>
-      </c>
-      <c r="BP7" s="1">
-        <v>100</v>
-      </c>
-      <c r="BQ7" s="1">
-        <v>100</v>
-      </c>
-      <c r="BR7" s="1">
-        <v>100</v>
-      </c>
-      <c r="BS7" s="1">
-        <v>100</v>
-      </c>
-      <c r="BT7" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="BU7" s="1">
         <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:73">
-      <c r="AR9" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2868,7 +2842,7 @@
         <v>39</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="AQ1" s="1" t="s">
         <v>42</v>
@@ -2948,13 +2922,13 @@
     </row>
     <row r="2" spans="1:67">
       <c r="A2" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>70</v>
@@ -2963,7 +2937,7 @@
         <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>72</v>
@@ -2975,7 +2949,7 @@
         <v>74</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>76</v>
@@ -2990,10 +2964,10 @@
         <v>79</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>80</v>
@@ -3020,7 +2994,7 @@
         <v>87</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>89</v>
@@ -3053,55 +3027,55 @@
         <v>5063159279999</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="AO2" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AP2" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AQ2" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AR2" s="1" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="AS2" t="s">
+        <v>104</v>
+      </c>
+      <c r="AT2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT2" s="1" t="s">
+      <c r="AU2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AU2" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="AV2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AW2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="AX2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AY2" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="AW2" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="AX2" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AY2" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="AZ2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BA2" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="BB2" s="1" t="s">
         <v>82</v>
@@ -3119,28 +3093,28 @@
         <v>100</v>
       </c>
       <c r="BG2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BH2" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="BH2" s="1" t="s">
+      <c r="BI2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BJ2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BK2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BL2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BM2" s="1">
+        <v>100</v>
+      </c>
+      <c r="BN2" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="BI2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BJ2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BK2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BL2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BM2" s="1">
-        <v>100</v>
-      </c>
-      <c r="BN2" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="BO2" s="1">
         <v>100</v>
@@ -3148,13 +3122,13 @@
     </row>
     <row r="3" spans="1:67">
       <c r="A3" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>70</v>
@@ -3163,7 +3137,7 @@
         <v>71</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>72</v>
@@ -3175,7 +3149,7 @@
         <v>74</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>76</v>
@@ -3190,10 +3164,10 @@
         <v>79</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>80</v>
@@ -3220,7 +3194,7 @@
         <v>87</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>89</v>
@@ -3253,37 +3227,37 @@
         <v>5063160372115</v>
       </c>
       <c r="AK3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AL3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AM3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AN3" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="AO3" s="1" t="s">
         <v>82</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AQ3" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AX3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AY3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AZ3" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="BA3" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="BB3" s="1" t="s">
         <v>82</v>
@@ -3301,10 +3275,10 @@
         <v>101</v>
       </c>
       <c r="BG3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BH3" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="BH3" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="BI3" s="1">
         <v>101</v>
@@ -3322,7 +3296,7 @@
         <v>101</v>
       </c>
       <c r="BN3" s="1" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="BO3" s="1">
         <v>101</v>

</xml_diff>